<commit_message>
Checkpoint before assistant change: Update test data used in the test generation process
Updates the glaucoma_test_results.xlsx file, likely to influence test point generation.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/glaucoma_test_results.xlsx
+++ b/glaucoma_test_results.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Pelli-Robinson" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="SPARCS" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Doctor Notes" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="humphrey_visual_field_24_2" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1235,4 +1236,106 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Patient Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Test Date</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Start Time</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>End Time</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Duration (seconds)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Total Points</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Correct Points</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Accuracy (%)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Doctor Notes</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Test Specific Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>kuti</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2025-05-28</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2025-05-28T05:16:46.587Z</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2025-05-28T05:19:38.077Z</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>171</v>
+      </c>
+      <c r="F2" t="n">
+        <v>54</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Checkpoint before assistant change: Update spreadsheet containing glaucoma test results with new data
Replace glaucoma_test_results.xlsx with a newer version reflecting updated test data.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/glaucoma_test_results.xlsx
+++ b/glaucoma_test_results.xlsx
@@ -16,6 +16,7 @@
     <sheet name="SPARCS" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Doctor Notes" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="humphrey_visual_field_24_2" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="unknown" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -548,6 +549,174 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Patient Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Test Date</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Start Time</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>End Time</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Duration (seconds)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Total Points</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Correct Points</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Accuracy (%)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Doctor Notes</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Test Specific Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ta</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2025-05-28</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>11:58:52 AM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>11:59:18 AM</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>26</v>
+      </c>
+      <c r="F2" t="n">
+        <v>72</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1.39</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ta</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2025-05-28</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>12:26:48 PM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>12:27:11 PM</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>23</v>
+      </c>
+      <c r="F3" t="n">
+        <v>72</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1.39</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ta</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2025-05-28</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1:10:12 PM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1:10:34 PM</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>22</v>
+      </c>
+      <c r="F4" t="n">
+        <v>72</v>
+      </c>
+      <c r="G4" t="n">
+        <v>6</v>
+      </c>
+      <c r="H4" t="n">
+        <v>8.33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Ensure consistent input for the contrast sensitivity test across all trials
Maintain active user input listener throughout CSV-1000 test trials by ensuring proper event listener handling and UI state reset after each response.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/glaucoma_test_results.xlsx
+++ b/glaucoma_test_results.xlsx
@@ -15,8 +15,6 @@
     <sheet name="Pelli-Robinson" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="SPARCS" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Doctor Notes" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="humphrey_visual_field_24_2" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="unknown" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -434,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -497,219 +495,6 @@
         <is>
           <t>Defects Detected</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>ANI</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2025-05-27</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2025-05-27T09:31:45.432Z</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2025-05-27T09:32:59.486Z</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>74</v>
-      </c>
-      <c r="F2" t="n">
-        <v>48</v>
-      </c>
-      <c r="G2" t="n">
-        <v>22</v>
-      </c>
-      <c r="H2" t="n">
-        <v>45.83</v>
-      </c>
-      <c r="J2" t="n">
-        <v>48</v>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>[{'pointIndex': 0, 'row': 0, 'col': 5, 'detected': True, 'reactionTime': 2632, 'timestamp': '2025-05-27T09:31:48.064Z'}, {'pointIndex': 1, 'row': 2, 'col': 5, 'detected': True, 'reactionTime': 1368, 'timestamp': '2025-05-27T09:31:49.944Z'}, {'pointIndex': 2, 'row': 2, 'col': 0, 'detected': False, 'reactionTime': 3000, 'timestamp': '2025-05-27T09:31:53.453Z'}, {'pointIndex': 3, 'row': 1, 'col': 6, 'detected': True, 'reactionTime': 1784, 'timestamp': '2025-05-27T09:31:55.746Z'}, {'pointIndex': 4, 'row': 5, 'col': 4, 'detected': True, 'reactionTime': 1856, 'timestamp': '2025-05-27T09:31:58.118Z'}, {'pointIndex': 5, 'row': 4, 'col': 3, 'detected': True, 'reactionTime': 1200, 'timestamp': '2025-05-27T09:31:59.831Z'}, {'pointIndex': 6, 'row': 0, 'col': 2, 'detected': True, 'reactionTime': 1316, 'timestamp': '2025-05-27T09:32:01.649Z'}, {'pointIndex': 7, 'row': 1, 'col': 1, 'detected': True, 'reactionTime': 1185, 'timestamp': '2025-05-27T09:32:03.344Z'}, {'pointIndex': 8, 'row': 3, 'col': 0, 'detected': True, 'reactionTime': 2535, 'timestamp': '2025-05-27T09:32:06.383Z'}, {'pointIndex': 9, 'row': 4, 'col': 6, 'detected': True, 'reactionTime': 1928, 'timestamp': '2025-05-27T09:32:08.816Z'}, {'pointIndex': 10, 'row': 1, 'col': 3, 'detected': True, 'reactionTime': 1656, 'timestamp': '2025-05-27T09:32:10.983Z'}, {'pointIndex': 11, 'row': 5, 'col': 2, 'detected': True, 'reactionTime': 1385, 'timestamp': '2025-05-27T09:32:12.883Z'}, {'pointIndex': 12, 'row': 1, 'col': 2, 'detected': True, 'reactionTime': 1139, 'timestamp': '2025-05-27T09:32:14.533Z'}, {'pointIndex': 13, 'row': 2, 'col': 7, 'detected': True, 'reactionTime': 1669, 'timestamp': '2025-05-27T09:32:16.714Z'}, {'pointIndex': 14, 'row': 1, 'col': 5, 'detected': True, 'reactionTime': 1116, 'timestamp': '2025-05-27T09:32:18.332Z'}, {'pointIndex': 15, 'row': 0, 'col': 5, 'detected': True, 'reactionTime': 1957, 'timestamp': '2025-05-27T09:32:20.799Z'}, {'pointIndex': 16, 'row': 5, 'col': 0, 'detected': True, 'reactionTime': 1701, 'timestamp': '2025-05-27T09:32:23.012Z'}, {'pointIndex': 17, 'row': 0, 'col': 1, 'detected': True, 'reactionTime': 1619, 'timestamp': '2025-05-27T09:32:25.131Z'}, {'pointIndex': 18, 'row': 4, 'col': 7, 'detected': True, 'reactionTime': 1590, 'timestamp': '2025-05-27T09:32:27.235Z'}, {'pointIndex': 19, 'row': 3, 'col': 5, 'detected': True, 'reactionTime': 1267, 'timestamp': '2025-05-27T09:32:29.018Z'}, {'pointIndex': 20, 'row': 3, 'col': 0, 'detected': False, 'reactionTime': 3000, 'timestamp': '2025-05-27T09:32:30.385Z'}, {'pointIndex': 21, 'row': 0, 'col': 2, 'detected': False, 'reactionTime': 3000, 'timestamp': '2025-05-27T09:32:30.940Z'}, {'pointIndex': 22, 'row': 5, 'col': 7, 'detected': False, 'reactionTime': 3000, 'timestamp': '2025-05-27T09:32:31.488Z'}, {'pointIndex': 23, 'row': 3, 'col': 2, 'detected': False, 'reactionTime': 3000, 'timestamp': '2025-05-27T09:32:32.101Z'}, {'pointIndex': 24, 'row': 2, 'col': 2, 'detected': False, 'reactionTime': 3000, 'timestamp': '2025-05-27T09:32:32.998Z'}, {'pointIndex': 25, 'row': 2, 'col': 7, 'detected': False, 'reactionTime': 3000, 'timestamp': '2025-05-27T09:32:33.640Z'}, {'pointIndex': 26, 'row': 0, 'col': 1, 'detected': False, 'reactionTime': 3000, 'timestamp': '2025-05-27T09:32:34.353Z'}, {'pointIndex': 27, 'row': 1, 'col': 6, 'detected': False, 'reactionTime': 3000, 'timestamp': '2025-05-27T09:32:37.882Z'}, {'pointIndex': 28, 'row': 5, 'col': 3, 'detected': True, 'reactionTime': 1304, 'timestamp': '2025-05-27T09:32:39.701Z'}, {'pointIndex': 29, 'row': 0, 'col': 3, 'detected': False, 'reactionTime': 3000, 'timestamp': '2025-05-27T09:32:40.707Z'}, {'pointIndex': 30, 'row': 2, 'col': 0, 'detected': False, 'reactionTime': 3000, 'timestamp': '2025-05-27T09:32:41.305Z'}, {'pointIndex': 31, 'row': 4, 'col': 3, 'detected': False, 'reactionTime': 3000, 'timestamp': '2025-05-27T09:32:41.882Z'}, {'pointIndex': 32, 'row': 5, 'col': 0, 'detected': False, 'reactionTime': 3000, 'timestamp': '2025-05-27T09:32:42.745Z'}, {'pointIndex': 33, 'row': 2, 'col': 5, 'detected': False, 'reactionTime': 3000, 'timestamp': '2025-05-27T09:32:43.322Z'}, {'pointIndex': 34, 'row': 1, 'col': 0, 'detected': False, 'reactionTime': 3000, 'timestamp': '2025-05-27T09:32:43.907Z'}, {'pointIndex': 35, 'row': 1, 'col': 5, 'detected': False, 'reactionTime': 3000, 'timestamp': '2025-05-27T09:32:44.448Z'}, {'pointIndex': 36, 'row': 4, 'col': 5, 'detected': False, 'reactionTime': 3000, 'timestamp': '2025-05-27T09:32:45.090Z'}, {'pointIndex': 37, 'row': 3, 'col': 3, 'detected': False, 'reactionTime': 3000, 'timestamp': '2025-05-27T09:32:45.746Z'}, {'pointIndex': 38, 'row': 5, 'col': 1, 'detected': False, 'reactionTime': 3000, 'timestamp': '2025-05-27T09:32:46.407Z'}, {'pointIndex': 39, 'row': 1, 'col': 5, 'detected': True, 'reactionTime': 1789, 'timestamp': '2025-05-27T09:32:48.703Z'}, {'pointIndex': 40, 'row': 5, 'col': 7, 'detected': True, 'reactionTime': 1444, 'timestamp': '2025-05-27T09:32:50.653Z'}, {'pointIndex': 41, 'row': 0, 'col': 7, 'detected': False, 'reactionTime': 921, 'timestamp': '2025-05-27T09:32:52.081Z'}, {'pointIndex': 42, 'row': 1, 'col': 5, 'detected': False, 'reactionTime': 857, 'timestamp': '2025-05-27T09:32:53.439Z'}, {'pointIndex': 43, 'row': 3, 'col': 1, 'detected': False, 'reactionTime': 524, 'timestamp': '2025-05-27T09:32:54.470Z'}, {'pointIndex': 44, 'row': 0, 'col': 0, 'detected': False, 'reactionTime': 701, 'timestamp': '2025-05-27T09:32:55.684Z'}, {'pointIndex': 45, 'row': 2, 'col': 6, 'detected': False, 'reactionTime': 3000, 'timestamp': '2025-05-27T09:32:57.621Z'}, {'pointIndex': 46, 'row': 3, 'col': 5, 'detected': False, 'reactionTime': 3000, 'timestamp': '2025-05-27T09:32:58.299Z'}, {'pointIndex': 47, 'row': 5, 'col': 0, 'detected': False, 'reactionTime': 3000, 'timestamp': '2025-05-27T09:32:58.983Z'}]</t>
-        </is>
-      </c>
-      <c r="L2" t="n">
-        <v>22</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Patient Name</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Test Date</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Start Time</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>End Time</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Duration (seconds)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Total Points</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Correct Points</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Accuracy (%)</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Doctor Notes</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Test Specific Data</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>ta</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2025-05-28</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>11:58:52 AM</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>11:59:18 AM</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>26</v>
-      </c>
-      <c r="F2" t="n">
-        <v>72</v>
-      </c>
-      <c r="G2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" t="n">
-        <v>1.39</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>ta</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2025-05-28</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>12:26:48 PM</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>12:27:11 PM</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>23</v>
-      </c>
-      <c r="F3" t="n">
-        <v>72</v>
-      </c>
-      <c r="G3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" t="n">
-        <v>1.39</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>ta</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2025-05-28</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1:10:12 PM</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>1:10:34 PM</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>22</v>
-      </c>
-      <c r="F4" t="n">
-        <v>72</v>
-      </c>
-      <c r="G4" t="n">
-        <v>6</v>
-      </c>
-      <c r="H4" t="n">
-        <v>8.33</v>
       </c>
     </row>
   </sheetData>
@@ -723,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -786,100 +571,6 @@
         <is>
           <t>Letter Accuracy</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>ANI</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2025-05-27</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2025-05-27T09:33:55.020Z</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2025-05-27T09:34:38.943Z</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>44</v>
-      </c>
-      <c r="F2" t="n">
-        <v>20</v>
-      </c>
-      <c r="G2" t="n">
-        <v>12</v>
-      </c>
-      <c r="H2" t="n">
-        <v>60</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>[100, 50, 25, 12.5, 6.25, 3.125, 1.56, 0.78, 0.39, 0.195]</t>
-        </is>
-      </c>
-      <c r="L2" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>ANI</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2025-05-27</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2025-05-27T15:09:35.311Z</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2025-05-27T15:10:04.946Z</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>30</v>
-      </c>
-      <c r="F3" t="n">
-        <v>20</v>
-      </c>
-      <c r="G3" t="n">
-        <v>13</v>
-      </c>
-      <c r="H3" t="n">
-        <v>65</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>[100, 50, 25, 12.5, 6.25, 3.125, 1.56, 0.78, 0.39, 0.195]</t>
-        </is>
-      </c>
-      <c r="L3" t="n">
-        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -1091,7 +782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1154,130 +845,6 @@
         <is>
           <t>Log Units</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>ANI</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2025-05-27</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2025-05-27T09:35:34.132Z</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2025-05-27T09:38:55.761Z</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>202</v>
-      </c>
-      <c r="F2" t="n">
-        <v>40</v>
-      </c>
-      <c r="G2" t="n">
-        <v>16</v>
-      </c>
-      <c r="H2" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>ANI</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2025-05-27</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>8:42:20 PM</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>8:44:21 PM</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>121</v>
-      </c>
-      <c r="F3" t="n">
-        <v>72</v>
-      </c>
-      <c r="G3" t="n">
-        <v>72</v>
-      </c>
-      <c r="H3" t="n">
-        <v>100</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>english</t>
-        </is>
-      </c>
-      <c r="K3" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="L3" t="n">
-        <v>1.15</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>ANI</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2025-05-27</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>8:51:46 PM</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>8:52:40 PM</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>54</v>
-      </c>
-      <c r="F4" t="n">
-        <v>72</v>
-      </c>
-      <c r="G4" t="n">
-        <v>72</v>
-      </c>
-      <c r="H4" t="n">
-        <v>100</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>english</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="L4" t="n">
-        <v>1.15</v>
       </c>
     </row>
   </sheetData>
@@ -1405,104 +972,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Patient Name</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Test Date</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Start Time</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>End Time</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Duration (seconds)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Total Points</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Correct Points</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Accuracy (%)</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Doctor Notes</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Test Specific Data</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>kuti</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2025-05-28</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2025-05-28T05:16:46.587Z</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2025-05-28T05:19:38.077Z</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>171</v>
-      </c>
-      <c r="F2" t="n">
-        <v>54</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add test results for glaucoma screening to the platform
Uploads the glaucoma_test_results_1748587757.xlsx file, which contains new glaucoma test results.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b1e33b71-088e-4faf-9a04-8015302ee74a
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: c7c812b6-e8e8-47cf-8e02-1cc251af9577
</commit_message>
<xml_diff>
--- a/glaucoma_test_results.xlsx
+++ b/glaucoma_test_results.xlsx
@@ -15,6 +15,8 @@
     <sheet name="Pelli-Robinson" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="SPARCS" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Doctor Notes" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="humphrey_visual_field_24_2" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="unknown" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -502,6 +504,106 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Patient Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Test Date</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Start Time</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>End Time</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Duration (seconds)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Total Points</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Correct Points</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Accuracy (%)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Doctor Notes</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Test Specific Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ta</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2025-06-27</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>12:15:34 AM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>12:21:40 AM</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>366</v>
+      </c>
+      <c r="F2" t="n">
+        <v>80</v>
+      </c>
+      <c r="G2" t="n">
+        <v>43</v>
+      </c>
+      <c r="H2" t="n">
+        <v>53.75</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -972,4 +1074,138 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Patient Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Test Date</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Start Time</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>End Time</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Duration (seconds)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Total Points</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Correct Points</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Accuracy (%)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Doctor Notes</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Test Specific Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ta</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2025-05-31</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2025-05-31T07:51:01.599Z</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2025-05-31T07:53:46.291Z</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>165</v>
+      </c>
+      <c r="F2" t="n">
+        <v>54</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ta</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2025-06-27</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2025-06-27T18:30:38.229Z</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2025-06-27T18:33:10.305Z</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>152</v>
+      </c>
+      <c r="F3" t="n">
+        <v>54</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>